<commit_message>
Plain-English site, benefit explainers and wave-2 official sources
Make the site readable for a layman: story homepage, out-of-every-£100,
per-person and per-household views, benefits explained one by one, glossary.
Add ONS population/households/GDP/PSF, OBR EFO, PESA UK-wide and Cabinet
Office spend parsers with trimmed fixtures, reconciliation rules R8-R14, and
fix the R7 memo-row bug. Review fixes: check-block aliases, lazy-loaded
provenance, cases-not-people wording, supplier name cleanup, docs updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/dwp/spring_forecast_2026.trimmed.xlsx
+++ b/tests/fixtures/dwp/spring_forecast_2026.trimmed.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Table 1a" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UK welfare " sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Table 1c" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="UK welfare " sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,6 +477,63 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Attendance Allowance</t>
+        </is>
+      </c>
+      <c r="BS7" t="n">
+        <v>5489.543391749996</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>6695.944034009999</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>8497.187075074615</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>9228.338202184894</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bereavement related benefits</t>
+        </is>
+      </c>
+      <c r="BS8" t="n">
+        <v>568.9204653500008</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>330.25930045</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>294.76084574215</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>276.444834413895</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Carer's Allowance</t>
+        </is>
+      </c>
+      <c r="BS9" t="n">
+        <v>2545.443967819999</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>3737.83555217</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>4580.463813760571</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>5024.566365170507</v>
+      </c>
+    </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
@@ -500,6 +558,25 @@
         <v>0</v>
       </c>
     </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Disability Living Allowance</t>
+        </is>
+      </c>
+      <c r="BS18" t="n">
+        <v>13233.12496869</v>
+      </c>
+      <c r="CA18" t="n">
+        <v>6862.28120161</v>
+      </c>
+      <c r="CC18" t="n">
+        <v>8289.471895168475</v>
+      </c>
+      <c r="CD18" t="n">
+        <v>8883.964483966784</v>
+      </c>
+    </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
@@ -567,6 +644,139 @@
         <v>31.57982987699923</v>
       </c>
     </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Housing benefits (exc. Universal Credit)</t>
+        </is>
+      </c>
+      <c r="BS29" t="n">
+        <v>24243.713647</v>
+      </c>
+      <c r="CA29" t="n">
+        <v>15772.59454746226</v>
+      </c>
+      <c r="CC29" t="n">
+        <v>12892.85164434135</v>
+      </c>
+      <c r="CD29" t="n">
+        <v>12474.2422992974</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Industrial injuries benefits in AME</t>
+        </is>
+      </c>
+      <c r="BS37" t="n">
+        <v>892.0474409811167</v>
+      </c>
+      <c r="CA37" t="n">
+        <v>735.7344942899998</v>
+      </c>
+      <c r="CC37" t="n">
+        <v>737.2787880313668</v>
+      </c>
+      <c r="CD37" t="n">
+        <v>732.0624524777965</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Jobseeker's Allowance</t>
+        </is>
+      </c>
+      <c r="BS41" t="n">
+        <v>2313.51601579</v>
+      </c>
+      <c r="CA41" t="n">
+        <v>313.2933446399999</v>
+      </c>
+      <c r="CC41" t="n">
+        <v>280.2886301077281</v>
+      </c>
+      <c r="CD41" t="n">
+        <v>365.8138756444606</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Maternity Allowance</t>
+        </is>
+      </c>
+      <c r="BS44" t="n">
+        <v>440.9409708199998</v>
+      </c>
+      <c r="CA44" t="n">
+        <v>412.1973994900001</v>
+      </c>
+      <c r="CC44" t="n">
+        <v>378.8690337763187</v>
+      </c>
+      <c r="CD44" t="n">
+        <v>403.5310375918293</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Pension Credit</t>
+        </is>
+      </c>
+      <c r="BS54" t="n">
+        <v>6078.706050869997</v>
+      </c>
+      <c r="CA54" t="n">
+        <v>5467.137915009998</v>
+      </c>
+      <c r="CC54" t="n">
+        <v>6144.472389476461</v>
+      </c>
+      <c r="CD54" t="n">
+        <v>6054.90028564646</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Personal Independence Payment</t>
+        </is>
+      </c>
+      <c r="BS55" t="n">
+        <v>3004.584281599999</v>
+      </c>
+      <c r="CA55" t="n">
+        <v>21668.78977710746</v>
+      </c>
+      <c r="CC55" t="n">
+        <v>28542.21737535933</v>
+      </c>
+      <c r="CD55" t="n">
+        <v>32100.18151294485</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Severe Disablement Allowance</t>
+        </is>
+      </c>
+      <c r="BS59" t="n">
+        <v>469.59270566</v>
+      </c>
+      <c r="CA59" t="n">
+        <v>56.45326820999999</v>
+      </c>
+      <c r="CC59" t="n">
+        <v>46.7605177230575</v>
+      </c>
+      <c r="CD59" t="n">
+        <v>41.99570652933794</v>
+      </c>
+    </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
@@ -634,6 +844,25 @@
         <v>243.0666327615986</v>
       </c>
     </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Statutory Maternity Pay</t>
+        </is>
+      </c>
+      <c r="BS67" t="n">
+        <v>2351</v>
+      </c>
+      <c r="CA67" t="n">
+        <v>2881</v>
+      </c>
+      <c r="CC67" t="n">
+        <v>3194.800881520547</v>
+      </c>
+      <c r="CD67" t="n">
+        <v>3316.841608693073</v>
+      </c>
+    </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
@@ -699,6 +928,25 @@
       </c>
       <c r="CD74" t="n">
         <v>15939.13811588398</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Winter Fuel Payments</t>
+        </is>
+      </c>
+      <c r="BS77" t="n">
+        <v>2073.16288804</v>
+      </c>
+      <c r="CA77" t="n">
+        <v>2031.926170666862</v>
+      </c>
+      <c r="CC77" t="n">
+        <v>1912.080880461916</v>
+      </c>
+      <c r="CD77" t="n">
+        <v>1911.382945820836</v>
       </c>
     </row>
     <row r="80">
@@ -795,6 +1043,481 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:CD63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Contents page</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Information relating to this table can be found in the 'Notes' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Spring Forecast</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Table 1c: Caseloads by benefit,</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>2015/16</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>2023/24</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>2025/26</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>thousands*</t>
+        </is>
+      </c>
+      <c r="BS3" t="inlineStr">
+        <is>
+          <t>Outturn</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>Outturn</t>
+        </is>
+      </c>
+      <c r="CC3" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+      <c r="CD3" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Attendance Allowance</t>
+        </is>
+      </c>
+      <c r="BS7" t="n">
+        <v>1603</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>1518</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>1775</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>1855</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS8" t="n">
+        <v>1459</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>1410</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>1662</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bereavement related benefits</t>
+        </is>
+      </c>
+      <c r="BS10" t="n">
+        <v>93</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>86</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>72</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Carer's Allowance</t>
+        </is>
+      </c>
+      <c r="BS11" t="n">
+        <v>1170</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>1258</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>1404</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS12" t="n">
+        <v>760</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>903</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>1018</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Disability Living Allowance</t>
+        </is>
+      </c>
+      <c r="BS20" t="n">
+        <v>3015</v>
+      </c>
+      <c r="CA20" t="n">
+        <v>1242</v>
+      </c>
+      <c r="CC20" t="n">
+        <v>1378</v>
+      </c>
+      <c r="CD20" t="n">
+        <v>1416</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS21" t="n">
+        <v>2989</v>
+      </c>
+      <c r="CA21" t="n">
+        <v>1232</v>
+      </c>
+      <c r="CC21" t="n">
+        <v>1370</v>
+      </c>
+      <c r="CD21" t="n">
+        <v>1409</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Employment and Support Allowance</t>
+        </is>
+      </c>
+      <c r="BS24" t="n">
+        <v>2356</v>
+      </c>
+      <c r="CA24" t="n">
+        <v>1573</v>
+      </c>
+      <c r="CC24" t="n">
+        <v>961</v>
+      </c>
+      <c r="CD24" t="n">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Housing benefits (exc. Universal Credit)</t>
+        </is>
+      </c>
+      <c r="BS30" t="n">
+        <v>4777</v>
+      </c>
+      <c r="CA30" t="n">
+        <v>2351</v>
+      </c>
+      <c r="CC30" t="n">
+        <v>1569</v>
+      </c>
+      <c r="CD30" t="n">
+        <v>1410</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Industrial Injuries benefits</t>
+        </is>
+      </c>
+      <c r="BS37" t="n">
+        <v>313</v>
+      </c>
+      <c r="CA37" t="n">
+        <v>215</v>
+      </c>
+      <c r="CC37" t="n">
+        <v>199</v>
+      </c>
+      <c r="CD37" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Jobseeker's Allowance</t>
+        </is>
+      </c>
+      <c r="BS41" t="n">
+        <v>652</v>
+      </c>
+      <c r="CA41" t="n">
+        <v>73</v>
+      </c>
+      <c r="CC41" t="n">
+        <v>57</v>
+      </c>
+      <c r="CD41" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Maternity Allowance</t>
+        </is>
+      </c>
+      <c r="BS46" t="n">
+        <v>62</v>
+      </c>
+      <c r="CA46" t="n">
+        <v>45</v>
+      </c>
+      <c r="CC46" t="n">
+        <v>39</v>
+      </c>
+      <c r="CD46" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Pension Credit</t>
+        </is>
+      </c>
+      <c r="BS50" t="n">
+        <v>2098</v>
+      </c>
+      <c r="CA50" t="n">
+        <v>1370</v>
+      </c>
+      <c r="CC50" t="n">
+        <v>1382</v>
+      </c>
+      <c r="CD50" t="n">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Personal Independence Payment</t>
+        </is>
+      </c>
+      <c r="BS51" t="n">
+        <v>594</v>
+      </c>
+      <c r="CA51" t="n">
+        <v>3198</v>
+      </c>
+      <c r="CC51" t="n">
+        <v>3878</v>
+      </c>
+      <c r="CD51" t="n">
+        <v>4193</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS52" t="n">
+        <v>588</v>
+      </c>
+      <c r="CA52" t="n">
+        <v>3163</v>
+      </c>
+      <c r="CC52" t="n">
+        <v>3836</v>
+      </c>
+      <c r="CD52" t="n">
+        <v>4147</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Severe Disablement Allowance</t>
+        </is>
+      </c>
+      <c r="BS54" t="n">
+        <v>113</v>
+      </c>
+      <c r="CA54" t="n">
+        <v>10</v>
+      </c>
+      <c r="CC54" t="n">
+        <v>8</v>
+      </c>
+      <c r="CD54" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>State Pension (includes contributory and non contributory)</t>
+        </is>
+      </c>
+      <c r="BS55" t="n">
+        <v>12957</v>
+      </c>
+      <c r="CA55" t="n">
+        <v>12776</v>
+      </c>
+      <c r="CC55" t="n">
+        <v>13204</v>
+      </c>
+      <c r="CD55" t="n">
+        <v>13220</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Statutory Maternity Pay</t>
+        </is>
+      </c>
+      <c r="BS56" t="n">
+        <v>264</v>
+      </c>
+      <c r="CA56" t="n">
+        <v>255</v>
+      </c>
+      <c r="CC56" t="n">
+        <v>264</v>
+      </c>
+      <c r="CD56" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Universal Credit</t>
+        </is>
+      </c>
+      <c r="BS58" t="n">
+        <v>130</v>
+      </c>
+      <c r="CA58" t="n">
+        <v>4706</v>
+      </c>
+      <c r="CC58" t="n">
+        <v>6404</v>
+      </c>
+      <c r="CD58" t="n">
+        <v>6807</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Winter Fuel Payments</t>
+        </is>
+      </c>
+      <c r="BS62" t="n">
+        <v>12215</v>
+      </c>
+      <c r="CA62" t="n">
+        <v>11626</v>
+      </c>
+      <c r="CC62" t="n">
+        <v>10891</v>
+      </c>
+      <c r="CD62" t="n">
+        <v>10845</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>* Summing the rows of caseloads for individual benefits to create a total caseload is not possible due to the overlap of individuals who are in receipt of more than one benefit.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:AI23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Plain-English site, benefit explainers and wave-2 official sources (#2)
Make the site readable for a layman: story homepage, out-of-every-£100,
per-person and per-household views, benefits explained one by one, glossary.
Add ONS population/households/GDP/PSF, OBR EFO, PESA UK-wide and Cabinet
Office spend parsers with trimmed fixtures, reconciliation rules R8-R14, and
fix the R7 memo-row bug. Review fixes: check-block aliases, lazy-loaded
provenance, cases-not-people wording, supplier name cleanup, docs updated.

Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/dwp/spring_forecast_2026.trimmed.xlsx
+++ b/tests/fixtures/dwp/spring_forecast_2026.trimmed.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Table 1a" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="UK welfare " sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Table 1c" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="UK welfare " sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,6 +477,63 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Attendance Allowance</t>
+        </is>
+      </c>
+      <c r="BS7" t="n">
+        <v>5489.543391749996</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>6695.944034009999</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>8497.187075074615</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>9228.338202184894</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bereavement related benefits</t>
+        </is>
+      </c>
+      <c r="BS8" t="n">
+        <v>568.9204653500008</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>330.25930045</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>294.76084574215</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>276.444834413895</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Carer's Allowance</t>
+        </is>
+      </c>
+      <c r="BS9" t="n">
+        <v>2545.443967819999</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>3737.83555217</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>4580.463813760571</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>5024.566365170507</v>
+      </c>
+    </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
@@ -500,6 +558,25 @@
         <v>0</v>
       </c>
     </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Disability Living Allowance</t>
+        </is>
+      </c>
+      <c r="BS18" t="n">
+        <v>13233.12496869</v>
+      </c>
+      <c r="CA18" t="n">
+        <v>6862.28120161</v>
+      </c>
+      <c r="CC18" t="n">
+        <v>8289.471895168475</v>
+      </c>
+      <c r="CD18" t="n">
+        <v>8883.964483966784</v>
+      </c>
+    </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
@@ -567,6 +644,139 @@
         <v>31.57982987699923</v>
       </c>
     </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Housing benefits (exc. Universal Credit)</t>
+        </is>
+      </c>
+      <c r="BS29" t="n">
+        <v>24243.713647</v>
+      </c>
+      <c r="CA29" t="n">
+        <v>15772.59454746226</v>
+      </c>
+      <c r="CC29" t="n">
+        <v>12892.85164434135</v>
+      </c>
+      <c r="CD29" t="n">
+        <v>12474.2422992974</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Industrial injuries benefits in AME</t>
+        </is>
+      </c>
+      <c r="BS37" t="n">
+        <v>892.0474409811167</v>
+      </c>
+      <c r="CA37" t="n">
+        <v>735.7344942899998</v>
+      </c>
+      <c r="CC37" t="n">
+        <v>737.2787880313668</v>
+      </c>
+      <c r="CD37" t="n">
+        <v>732.0624524777965</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Jobseeker's Allowance</t>
+        </is>
+      </c>
+      <c r="BS41" t="n">
+        <v>2313.51601579</v>
+      </c>
+      <c r="CA41" t="n">
+        <v>313.2933446399999</v>
+      </c>
+      <c r="CC41" t="n">
+        <v>280.2886301077281</v>
+      </c>
+      <c r="CD41" t="n">
+        <v>365.8138756444606</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Maternity Allowance</t>
+        </is>
+      </c>
+      <c r="BS44" t="n">
+        <v>440.9409708199998</v>
+      </c>
+      <c r="CA44" t="n">
+        <v>412.1973994900001</v>
+      </c>
+      <c r="CC44" t="n">
+        <v>378.8690337763187</v>
+      </c>
+      <c r="CD44" t="n">
+        <v>403.5310375918293</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Pension Credit</t>
+        </is>
+      </c>
+      <c r="BS54" t="n">
+        <v>6078.706050869997</v>
+      </c>
+      <c r="CA54" t="n">
+        <v>5467.137915009998</v>
+      </c>
+      <c r="CC54" t="n">
+        <v>6144.472389476461</v>
+      </c>
+      <c r="CD54" t="n">
+        <v>6054.90028564646</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Personal Independence Payment</t>
+        </is>
+      </c>
+      <c r="BS55" t="n">
+        <v>3004.584281599999</v>
+      </c>
+      <c r="CA55" t="n">
+        <v>21668.78977710746</v>
+      </c>
+      <c r="CC55" t="n">
+        <v>28542.21737535933</v>
+      </c>
+      <c r="CD55" t="n">
+        <v>32100.18151294485</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Severe Disablement Allowance</t>
+        </is>
+      </c>
+      <c r="BS59" t="n">
+        <v>469.59270566</v>
+      </c>
+      <c r="CA59" t="n">
+        <v>56.45326820999999</v>
+      </c>
+      <c r="CC59" t="n">
+        <v>46.7605177230575</v>
+      </c>
+      <c r="CD59" t="n">
+        <v>41.99570652933794</v>
+      </c>
+    </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
@@ -634,6 +844,25 @@
         <v>243.0666327615986</v>
       </c>
     </row>
+    <row r="67">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Statutory Maternity Pay</t>
+        </is>
+      </c>
+      <c r="BS67" t="n">
+        <v>2351</v>
+      </c>
+      <c r="CA67" t="n">
+        <v>2881</v>
+      </c>
+      <c r="CC67" t="n">
+        <v>3194.800881520547</v>
+      </c>
+      <c r="CD67" t="n">
+        <v>3316.841608693073</v>
+      </c>
+    </row>
     <row r="72">
       <c r="B72" t="inlineStr">
         <is>
@@ -699,6 +928,25 @@
       </c>
       <c r="CD74" t="n">
         <v>15939.13811588398</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Winter Fuel Payments</t>
+        </is>
+      </c>
+      <c r="BS77" t="n">
+        <v>2073.16288804</v>
+      </c>
+      <c r="CA77" t="n">
+        <v>2031.926170666862</v>
+      </c>
+      <c r="CC77" t="n">
+        <v>1912.080880461916</v>
+      </c>
+      <c r="CD77" t="n">
+        <v>1911.382945820836</v>
       </c>
     </row>
     <row r="80">
@@ -795,6 +1043,481 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:CD63"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Contents page</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Information relating to this table can be found in the 'Notes' tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Spring Forecast</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Table 1c: Caseloads by benefit,</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>2015/16</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>2023/24</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>2025/26</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>2026/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>thousands*</t>
+        </is>
+      </c>
+      <c r="BS3" t="inlineStr">
+        <is>
+          <t>Outturn</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>Outturn</t>
+        </is>
+      </c>
+      <c r="CC3" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+      <c r="CD3" t="inlineStr">
+        <is>
+          <t>Forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Attendance Allowance</t>
+        </is>
+      </c>
+      <c r="BS7" t="n">
+        <v>1603</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>1518</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>1775</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>1855</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS8" t="n">
+        <v>1459</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>1410</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>1662</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bereavement related benefits</t>
+        </is>
+      </c>
+      <c r="BS10" t="n">
+        <v>93</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>86</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>72</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Carer's Allowance</t>
+        </is>
+      </c>
+      <c r="BS11" t="n">
+        <v>1170</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>1258</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>1404</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS12" t="n">
+        <v>760</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>903</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>1018</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Disability Living Allowance</t>
+        </is>
+      </c>
+      <c r="BS20" t="n">
+        <v>3015</v>
+      </c>
+      <c r="CA20" t="n">
+        <v>1242</v>
+      </c>
+      <c r="CC20" t="n">
+        <v>1378</v>
+      </c>
+      <c r="CD20" t="n">
+        <v>1416</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS21" t="n">
+        <v>2989</v>
+      </c>
+      <c r="CA21" t="n">
+        <v>1232</v>
+      </c>
+      <c r="CC21" t="n">
+        <v>1370</v>
+      </c>
+      <c r="CD21" t="n">
+        <v>1409</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Employment and Support Allowance</t>
+        </is>
+      </c>
+      <c r="BS24" t="n">
+        <v>2356</v>
+      </c>
+      <c r="CA24" t="n">
+        <v>1573</v>
+      </c>
+      <c r="CC24" t="n">
+        <v>961</v>
+      </c>
+      <c r="CD24" t="n">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Housing benefits (exc. Universal Credit)</t>
+        </is>
+      </c>
+      <c r="BS30" t="n">
+        <v>4777</v>
+      </c>
+      <c r="CA30" t="n">
+        <v>2351</v>
+      </c>
+      <c r="CC30" t="n">
+        <v>1569</v>
+      </c>
+      <c r="CD30" t="n">
+        <v>1410</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Industrial Injuries benefits</t>
+        </is>
+      </c>
+      <c r="BS37" t="n">
+        <v>313</v>
+      </c>
+      <c r="CA37" t="n">
+        <v>215</v>
+      </c>
+      <c r="CC37" t="n">
+        <v>199</v>
+      </c>
+      <c r="CD37" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Jobseeker's Allowance</t>
+        </is>
+      </c>
+      <c r="BS41" t="n">
+        <v>652</v>
+      </c>
+      <c r="CA41" t="n">
+        <v>73</v>
+      </c>
+      <c r="CC41" t="n">
+        <v>57</v>
+      </c>
+      <c r="CD41" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Maternity Allowance</t>
+        </is>
+      </c>
+      <c r="BS46" t="n">
+        <v>62</v>
+      </c>
+      <c r="CA46" t="n">
+        <v>45</v>
+      </c>
+      <c r="CC46" t="n">
+        <v>39</v>
+      </c>
+      <c r="CD46" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Pension Credit</t>
+        </is>
+      </c>
+      <c r="BS50" t="n">
+        <v>2098</v>
+      </c>
+      <c r="CA50" t="n">
+        <v>1370</v>
+      </c>
+      <c r="CC50" t="n">
+        <v>1382</v>
+      </c>
+      <c r="CD50" t="n">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Personal Independence Payment</t>
+        </is>
+      </c>
+      <c r="BS51" t="n">
+        <v>594</v>
+      </c>
+      <c r="CA51" t="n">
+        <v>3198</v>
+      </c>
+      <c r="CC51" t="n">
+        <v>3878</v>
+      </c>
+      <c r="CD51" t="n">
+        <v>4193</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>of which in payment</t>
+        </is>
+      </c>
+      <c r="BS52" t="n">
+        <v>588</v>
+      </c>
+      <c r="CA52" t="n">
+        <v>3163</v>
+      </c>
+      <c r="CC52" t="n">
+        <v>3836</v>
+      </c>
+      <c r="CD52" t="n">
+        <v>4147</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Severe Disablement Allowance</t>
+        </is>
+      </c>
+      <c r="BS54" t="n">
+        <v>113</v>
+      </c>
+      <c r="CA54" t="n">
+        <v>10</v>
+      </c>
+      <c r="CC54" t="n">
+        <v>8</v>
+      </c>
+      <c r="CD54" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>State Pension (includes contributory and non contributory)</t>
+        </is>
+      </c>
+      <c r="BS55" t="n">
+        <v>12957</v>
+      </c>
+      <c r="CA55" t="n">
+        <v>12776</v>
+      </c>
+      <c r="CC55" t="n">
+        <v>13204</v>
+      </c>
+      <c r="CD55" t="n">
+        <v>13220</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Statutory Maternity Pay</t>
+        </is>
+      </c>
+      <c r="BS56" t="n">
+        <v>264</v>
+      </c>
+      <c r="CA56" t="n">
+        <v>255</v>
+      </c>
+      <c r="CC56" t="n">
+        <v>264</v>
+      </c>
+      <c r="CD56" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Universal Credit</t>
+        </is>
+      </c>
+      <c r="BS58" t="n">
+        <v>130</v>
+      </c>
+      <c r="CA58" t="n">
+        <v>4706</v>
+      </c>
+      <c r="CC58" t="n">
+        <v>6404</v>
+      </c>
+      <c r="CD58" t="n">
+        <v>6807</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Winter Fuel Payments</t>
+        </is>
+      </c>
+      <c r="BS62" t="n">
+        <v>12215</v>
+      </c>
+      <c r="CA62" t="n">
+        <v>11626</v>
+      </c>
+      <c r="CC62" t="n">
+        <v>10891</v>
+      </c>
+      <c r="CD62" t="n">
+        <v>10845</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>* Summing the rows of caseloads for individual benefits to create a total caseload is not possible due to the overlap of individuals who are in receipt of more than one benefit.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:AI23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>